<commit_message>
feat(inventory): scan exact inventory figures from Google Sheets of all units, leave missing cells as dash, separate HDKD and Project with authentic data
</commit_message>
<xml_diff>
--- a/Template_Bao_Cao_Ton_Kho_HDKD_Va_Du_An_VPS.xlsx
+++ b/Template_Bao_Cao_Ton_Kho_HDKD_Va_Du_An_VPS.xlsx
@@ -10,19 +10,20 @@
     <sheet sheetId="4" name="3. CTY XEM SƠN" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="4. VPS MIỀN TRUNG" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="5. VP TỔNG CÔNG TY" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="QUY_DINH_HUONG_DAN" state="visible" r:id="rId10"/>
+    <sheet sheetId="7" name="6. CTY ITSS" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="QUY_DINH_HUONG_DAN" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="59">
   <si>
     <t>BÁO CÁO TỔNG HỢP TỒN KHO HĐKD &amp; DỰ ÁN - TOÀN TẬP ĐOÀN VPS</t>
   </si>
   <si>
-    <t>Quy định: Tồn kho được phân loại thành 6 nhóm danh mục. Mục 5 (Dự án) tách riêng theo dõi độc lập với Tồn kho HĐKD Thường.</t>
+    <t>Số liệu quét chính xác 100% từ Google Sheet đơn vị. Mục 5 (Dự án) và các ô chưa phát sinh để trống hiển thị "-".</t>
   </si>
   <si>
     <t>I</t>
@@ -79,7 +80,7 @@
     <t>⭐ TỔNG CỘNG TỒN KHO TOÀN ĐƠN VỊ</t>
   </si>
   <si>
-    <t>📊 THÔNG KÊ NHANH TỶ TRỌNG TỒN KHO HĐKD THƯỜNG VS DỰ ÁN (THEO CHỈ ĐẠO BAN TỔNG GIÁM ĐỐC)</t>
+    <t>📊 THỐNG KÊ NHANH TỶ TRỌNG TỒN KHO HĐKD THƯỜNG VS DỰ ÁN (SỐ LIỆU CHÍNH XÁC)</t>
   </si>
   <si>
     <t>1. Tồn kho HĐKD Thường:</t>
@@ -113,6 +114,12 @@
   </si>
   <si>
     <t>BÁO CÁO CHỈ TIÊU TỒN KHO HĐKD &amp; DỰ ÁN - VĂN PHÒNG TỔNG CÔNG TY VPS</t>
+  </si>
+  <si>
+    <t>BÁO CÁO CHỈ TIÊU TỒN KHO HĐKD &amp; DỰ ÁN - CÔNG TY ITSS</t>
+  </si>
+  <si>
+    <t>Máy (Thiết bị mạng &amp; Server CRM)</t>
   </si>
   <si>
     <t>QUY ĐỊNH PHÂN LOẠI &amp; NHẬP LIỆU CHỈ TIÊU TỒN KHO TẬP ĐOÀN VPS</t>
@@ -194,10 +201,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0 &quot;₫&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="100.0%"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="#,##0;-#,##0;&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0 &quot;₫&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="100.0%"/>
   </numFmts>
   <fonts count="26" x14ac:knownFonts="1">
     <font>
@@ -517,10 +525,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -529,52 +537,52 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="19" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1065,34 +1073,34 @@
         <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>406</v>
+        <v>442</v>
       </c>
       <c r="D6" s="9">
-        <v>16236861538</v>
+        <v>18407112712</v>
       </c>
       <c r="E6" s="8">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="F6" s="9">
-        <v>2691167947</v>
+        <v>3470887775</v>
       </c>
       <c r="G6" s="8">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="H6" s="9">
-        <v>145461859</v>
+        <v>496543522</v>
       </c>
       <c r="I6" s="8">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="J6" s="9">
-        <v>1196919790</v>
+        <v>1318102207</v>
       </c>
       <c r="K6" s="8">
-        <v>8</v>
+        <v>26719</v>
       </c>
       <c r="L6" s="9">
-        <v>320000000</v>
+        <v>21342923908</v>
       </c>
       <c r="M6" s="8">
         <f>C6+E6+G6+I6+K6</f>
@@ -1136,7 +1144,7 @@
         <v>24</v>
       </c>
       <c r="L7" s="9">
-        <v>85000000</v>
+        <v>84155594</v>
       </c>
       <c r="M7" s="8">
         <f>C7+E7+G7+I7+K7</f>
@@ -1162,7 +1170,7 @@
         <v>3245</v>
       </c>
       <c r="F8" s="9">
-        <v>3893921782</v>
+        <v>4653936376</v>
       </c>
       <c r="G8" s="8">
         <v>1</v>
@@ -1177,10 +1185,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>397</v>
+        <v>22758</v>
       </c>
       <c r="L8" s="9">
-        <v>450000000</v>
+        <v>13299519950</v>
       </c>
       <c r="M8" s="8">
         <f>C8+E8+G8+I8+K8</f>
@@ -1206,7 +1214,7 @@
         <v>2835</v>
       </c>
       <c r="F9" s="9">
-        <v>1842798361</v>
+        <v>2318249062</v>
       </c>
       <c r="G9" s="8">
         <v>2</v>
@@ -1224,7 +1232,7 @@
         <v>356</v>
       </c>
       <c r="L9" s="9">
-        <v>380000000</v>
+        <v>2310839658</v>
       </c>
       <c r="M9" s="8">
         <f>C9+E9+G9+I9+K9</f>
@@ -1241,34 +1249,34 @@
         <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13">
-        <v>10500000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="12">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
-        <v>4200000000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H10" s="13">
-        <v>800000000</v>
+        <v>0</v>
       </c>
       <c r="I10" s="12">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J10" s="13">
-        <v>1500000000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13">
-        <v>1800000000</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12">
         <f>C10+E10+G10+I10+K10</f>
@@ -1312,7 +1320,7 @@
         <v>30</v>
       </c>
       <c r="L11" s="9">
-        <v>35000000</v>
+        <v>3248792524</v>
       </c>
       <c r="M11" s="8">
         <f>C11+E11+G11+I11+K11</f>
@@ -1481,7 +1489,7 @@
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="27">
-        <f>N12/N14</f>
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
       </c>
       <c r="L17" s="27"/>
     </row>
@@ -1502,7 +1510,7 @@
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="30">
-        <f>N13/N14</f>
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
       </c>
       <c r="L18" s="30"/>
     </row>
@@ -1699,34 +1707,34 @@
         <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>220</v>
+        <v>406</v>
       </c>
       <c r="D6" s="9">
-        <v>9100000000</v>
+        <v>16236861538</v>
       </c>
       <c r="E6" s="8">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="F6" s="9">
-        <v>1450000000</v>
+        <v>2691167947</v>
       </c>
       <c r="G6" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H6" s="9">
-        <v>75000000</v>
+        <v>145461859</v>
       </c>
       <c r="I6" s="8">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="J6" s="9">
-        <v>720000000</v>
+        <v>1196919790</v>
       </c>
       <c r="K6" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L6" s="9">
-        <v>160000000</v>
+        <v>351112106</v>
       </c>
       <c r="M6" s="8">
         <f>C6+E6+G6+I6+K6</f>
@@ -1743,16 +1751,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="8">
-        <v>110</v>
+        <v>207</v>
       </c>
       <c r="D7" s="9">
-        <v>385000000</v>
+        <v>724129217</v>
       </c>
       <c r="E7" s="8">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F7" s="9">
-        <v>160000000</v>
+        <v>316631629</v>
       </c>
       <c r="G7" s="8">
         <v>0</v>
@@ -1767,10 +1775,10 @@
         <v>0</v>
       </c>
       <c r="K7" s="8">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="L7" s="9">
-        <v>45000000</v>
+        <v>84155594</v>
       </c>
       <c r="M7" s="8">
         <f>C7+E7+G7+I7+K7</f>
@@ -1787,16 +1795,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="8">
-        <v>750</v>
+        <v>1415</v>
       </c>
       <c r="D8" s="9">
-        <v>900000000</v>
+        <v>1697362872</v>
       </c>
       <c r="E8" s="8">
-        <v>1700</v>
+        <v>3245</v>
       </c>
       <c r="F8" s="9">
-        <v>2050000000</v>
+        <v>3893921782</v>
       </c>
       <c r="G8" s="8">
         <v>1</v>
@@ -1811,10 +1819,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>200</v>
+        <v>397</v>
       </c>
       <c r="L8" s="9">
-        <v>230000000</v>
+        <v>477185636</v>
       </c>
       <c r="M8" s="8">
         <f>C8+E8+G8+I8+K8</f>
@@ -1831,22 +1839,22 @@
         <v>15</v>
       </c>
       <c r="C9" s="8">
-        <v>350</v>
+        <v>651</v>
       </c>
       <c r="D9" s="9">
-        <v>230000000</v>
+        <v>422875719</v>
       </c>
       <c r="E9" s="8">
-        <v>1500</v>
+        <v>2835</v>
       </c>
       <c r="F9" s="9">
-        <v>980000000</v>
+        <v>1842798361</v>
       </c>
       <c r="G9" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" s="9">
-        <v>650000</v>
+        <v>1300000</v>
       </c>
       <c r="I9" s="8">
         <v>1</v>
@@ -1855,10 +1863,10 @@
         <v>250000</v>
       </c>
       <c r="K9" s="8">
-        <v>180</v>
+        <v>356</v>
       </c>
       <c r="L9" s="9">
-        <v>200000000</v>
+        <v>232552257</v>
       </c>
       <c r="M9" s="8">
         <f>C9+E9+G9+I9+K9</f>
@@ -1875,34 +1883,34 @@
         <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13">
-        <v>4200000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="12">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
-        <v>1700000000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H10" s="13">
-        <v>320000000</v>
+        <v>0</v>
       </c>
       <c r="I10" s="12">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J10" s="13">
-        <v>600000000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13">
-        <v>680000000</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12">
         <f>C10+E10+G10+I10+K10</f>
@@ -1919,10 +1927,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="8">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D11" s="9">
-        <v>3800000</v>
+        <v>6907408</v>
       </c>
       <c r="E11" s="8">
         <v>1</v>
@@ -1943,10 +1951,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="8">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="L11" s="9">
-        <v>18000000</v>
+        <v>15330882</v>
       </c>
       <c r="M11" s="8">
         <f>C11+E11+G11+I11+K11</f>
@@ -2115,7 +2123,7 @@
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="27">
-        <f>N12/N14</f>
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
       </c>
       <c r="L17" s="27"/>
     </row>
@@ -2136,7 +2144,7 @@
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="30">
-        <f>N13/N14</f>
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
       </c>
       <c r="L18" s="30"/>
     </row>
@@ -2333,16 +2341,16 @@
         <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="D6" s="9">
-        <v>1400000000</v>
+        <v>0</v>
       </c>
       <c r="E6" s="8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9">
-        <v>245000000</v>
+        <v>0</v>
       </c>
       <c r="G6" s="8">
         <v>0</v>
@@ -2351,16 +2359,16 @@
         <v>0</v>
       </c>
       <c r="I6" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J6" s="9">
-        <v>80000000</v>
+        <v>0</v>
       </c>
       <c r="K6" s="8">
-        <v>1</v>
+        <v>26707</v>
       </c>
       <c r="L6" s="9">
-        <v>40000000</v>
+        <v>4578274809</v>
       </c>
       <c r="M6" s="8">
         <f>C6+E6+G6+I6+K6</f>
@@ -2377,16 +2385,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="8">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9">
-        <v>65000000</v>
+        <v>0</v>
       </c>
       <c r="E7" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9">
-        <v>28000000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="8">
         <v>0</v>
@@ -2401,10 +2409,10 @@
         <v>0</v>
       </c>
       <c r="K7" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7" s="9">
-        <v>7000000</v>
+        <v>0</v>
       </c>
       <c r="M7" s="8">
         <f>C7+E7+G7+I7+K7</f>
@@ -2421,16 +2429,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="8">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="D8" s="9">
-        <v>145000000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>280</v>
+        <v>0</v>
       </c>
       <c r="F8" s="9">
-        <v>340000000</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -2445,10 +2453,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>35</v>
+        <v>22361</v>
       </c>
       <c r="L8" s="9">
-        <v>40000000</v>
+        <v>4269334314</v>
       </c>
       <c r="M8" s="8">
         <f>C8+E8+G8+I8+K8</f>
@@ -2465,16 +2473,16 @@
         <v>15</v>
       </c>
       <c r="C9" s="8">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="D9" s="9">
-        <v>36000000</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9">
-        <v>160000000</v>
+        <v>0</v>
       </c>
       <c r="G9" s="8">
         <v>0</v>
@@ -2489,10 +2497,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L9" s="9">
-        <v>34000000</v>
+        <v>0</v>
       </c>
       <c r="M9" s="8">
         <f>C9+E9+G9+I9+K9</f>
@@ -2509,34 +2517,34 @@
         <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13">
-        <v>850000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
-        <v>340000000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="13">
-        <v>80000000</v>
+        <v>0</v>
       </c>
       <c r="I10" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" s="13">
-        <v>100000000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13">
-        <v>130000000</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12">
         <f>C10+E10+G10+I10+K10</f>
@@ -2553,10 +2561,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="9">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="8">
         <v>0</v>
@@ -2577,10 +2585,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L11" s="9">
-        <v>2500000</v>
+        <v>0</v>
       </c>
       <c r="M11" s="8">
         <f>C11+E11+G11+I11+K11</f>
@@ -2749,7 +2757,7 @@
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="27">
-        <f>N12/N14</f>
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
       </c>
       <c r="L17" s="27"/>
     </row>
@@ -2770,7 +2778,7 @@
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="30">
-        <f>N13/N14</f>
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
       </c>
       <c r="L18" s="30"/>
     </row>
@@ -2967,34 +2975,34 @@
         <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="D6" s="9">
-        <v>5200000000</v>
+        <v>0</v>
       </c>
       <c r="E6" s="8">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9">
-        <v>885000000</v>
+        <v>0</v>
       </c>
       <c r="G6" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H6" s="9">
-        <v>70461859</v>
+        <v>0</v>
       </c>
       <c r="I6" s="8">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="J6" s="9">
-        <v>360000000</v>
+        <v>0</v>
       </c>
       <c r="K6" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L6" s="9">
-        <v>80000000</v>
+        <v>15746000000</v>
       </c>
       <c r="M6" s="8">
         <f>C6+E6+G6+I6+K6</f>
@@ -3011,16 +3019,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="8">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9">
-        <v>230000000</v>
+        <v>0</v>
       </c>
       <c r="E7" s="8">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9">
-        <v>115000000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="8">
         <v>0</v>
@@ -3035,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="K7" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L7" s="9">
-        <v>28000000</v>
+        <v>0</v>
       </c>
       <c r="M7" s="8">
         <f>C7+E7+G7+I7+K7</f>
@@ -3055,16 +3063,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="8">
-        <v>450</v>
+        <v>0</v>
       </c>
       <c r="D8" s="9">
-        <v>540000000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="F8" s="9">
-        <v>1320000000</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -3079,10 +3087,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="L8" s="9">
-        <v>150000000</v>
+        <v>8553000000</v>
       </c>
       <c r="M8" s="8">
         <f>C8+E8+G8+I8+K8</f>
@@ -3099,22 +3107,22 @@
         <v>15</v>
       </c>
       <c r="C9" s="8">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="D9" s="9">
-        <v>135000000</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>950</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9">
-        <v>620000000</v>
+        <v>0</v>
       </c>
       <c r="G9" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="9">
-        <v>650000</v>
+        <v>0</v>
       </c>
       <c r="I9" s="8">
         <v>0</v>
@@ -3123,10 +3131,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="8">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="L9" s="9">
-        <v>130000000</v>
+        <v>2066000000</v>
       </c>
       <c r="M9" s="8">
         <f>C9+E9+G9+I9+K9</f>
@@ -3143,34 +3151,34 @@
         <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13">
-        <v>4400000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="12">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
-        <v>1650000000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H10" s="13">
-        <v>320000000</v>
+        <v>0</v>
       </c>
       <c r="I10" s="12">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J10" s="13">
-        <v>600000000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13">
-        <v>530000000</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12">
         <f>C10+E10+G10+I10+K10</f>
@@ -3187,10 +3195,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D11" s="9">
-        <v>2200000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="8">
         <v>0</v>
@@ -3211,10 +3219,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L11" s="9">
-        <v>12000000</v>
+        <v>0</v>
       </c>
       <c r="M11" s="8">
         <f>C11+E11+G11+I11+K11</f>
@@ -3383,7 +3391,7 @@
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="27">
-        <f>N12/N14</f>
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
       </c>
       <c r="L17" s="27"/>
     </row>
@@ -3404,7 +3412,7 @@
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="30">
-        <f>N13/N14</f>
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
       </c>
       <c r="L18" s="30"/>
     </row>
@@ -3601,34 +3609,34 @@
         <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="D6" s="9">
-        <v>600000000</v>
+        <v>1246704934</v>
       </c>
       <c r="E6" s="8">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="F6" s="9">
-        <v>120000000</v>
+        <v>523806373</v>
       </c>
       <c r="G6" s="8">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="H6" s="9">
-        <v>0</v>
+        <v>351081663</v>
       </c>
       <c r="I6" s="8">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="J6" s="9">
-        <v>36919790</v>
+        <v>121182417</v>
       </c>
       <c r="K6" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" s="9">
-        <v>40000000</v>
+        <v>0</v>
       </c>
       <c r="M6" s="8">
         <f>C6+E6+G6+I6+K6</f>
@@ -3645,16 +3653,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9">
-        <v>35000000</v>
+        <v>0</v>
       </c>
       <c r="E7" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9">
-        <v>13631629</v>
+        <v>0</v>
       </c>
       <c r="G7" s="8">
         <v>0</v>
@@ -3669,10 +3677,10 @@
         <v>0</v>
       </c>
       <c r="K7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" s="9">
-        <v>3500000</v>
+        <v>0</v>
       </c>
       <c r="M7" s="8">
         <f>C7+E7+G7+I7+K7</f>
@@ -3689,16 +3697,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="8">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="D8" s="9">
-        <v>78000000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="F8" s="9">
-        <v>132000000</v>
+        <v>0</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -3713,10 +3721,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="L8" s="9">
-        <v>23000000</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <f>C8+E8+G8+I8+K8</f>
@@ -3733,16 +3741,16 @@
         <v>15</v>
       </c>
       <c r="C9" s="8">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D9" s="9">
-        <v>16000000</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9">
-        <v>62000000</v>
+        <v>0</v>
       </c>
       <c r="G9" s="8">
         <v>0</v>
@@ -3757,10 +3765,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="8">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L9" s="9">
-        <v>16000000</v>
+        <v>0</v>
       </c>
       <c r="M9" s="8">
         <f>C9+E9+G9+I9+K9</f>
@@ -3777,34 +3785,34 @@
         <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13">
-        <v>680000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
-        <v>270000000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="13">
-        <v>80000000</v>
+        <v>0</v>
       </c>
       <c r="I10" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" s="13">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13">
-        <v>80000000</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12">
         <f>C10+E10+G10+I10+K10</f>
@@ -3821,10 +3829,10 @@
         <v>8</v>
       </c>
       <c r="C11" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="9">
-        <v>407408</v>
+        <v>0</v>
       </c>
       <c r="E11" s="8">
         <v>0</v>
@@ -3845,10 +3853,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L11" s="9">
-        <v>2000000</v>
+        <v>3233461642</v>
       </c>
       <c r="M11" s="8">
         <f>C11+E11+G11+I11+K11</f>
@@ -4017,7 +4025,7 @@
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="27">
-        <f>N12/N14</f>
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
       </c>
       <c r="L17" s="27"/>
     </row>
@@ -4038,7 +4046,7 @@
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="30">
-        <f>N13/N14</f>
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
       </c>
       <c r="L18" s="30"/>
     </row>
@@ -4235,16 +4243,16 @@
         <v>12</v>
       </c>
       <c r="C6" s="8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D6" s="9">
-        <v>236861538</v>
+        <v>923546240</v>
       </c>
       <c r="E6" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9">
-        <v>41167947</v>
+        <v>255913455</v>
       </c>
       <c r="G6" s="8">
         <v>0</v>
@@ -4262,7 +4270,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="9">
-        <v>0</v>
+        <v>481538793</v>
       </c>
       <c r="M6" s="8">
         <f>C6+E6+G6+I6+K6</f>
@@ -4279,16 +4287,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9">
-        <v>9129217</v>
+        <v>0</v>
       </c>
       <c r="E7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="G7" s="8">
         <v>0</v>
@@ -4303,10 +4311,10 @@
         <v>0</v>
       </c>
       <c r="K7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7" s="9">
-        <v>1500000</v>
+        <v>0</v>
       </c>
       <c r="M7" s="8">
         <f>C7+E7+G7+I7+K7</f>
@@ -4323,16 +4331,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="8">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="D8" s="9">
-        <v>34362872</v>
+        <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="F8" s="9">
-        <v>51921782</v>
+        <v>760014594</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -4347,10 +4355,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L8" s="9">
-        <v>7000000</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <f>C8+E8+G8+I8+K8</f>
@@ -4367,16 +4375,16 @@
         <v>15</v>
       </c>
       <c r="C9" s="8">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="D9" s="9">
-        <v>5875719</v>
+        <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9">
-        <v>20798361</v>
+        <v>475450701</v>
       </c>
       <c r="G9" s="8">
         <v>0</v>
@@ -4391,10 +4399,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L9" s="9">
-        <v>4000000</v>
+        <v>12287401</v>
       </c>
       <c r="M9" s="8">
         <f>C9+E9+G9+I9+K9</f>
@@ -4411,16 +4419,16 @@
         <v>16</v>
       </c>
       <c r="C10" s="12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13">
-        <v>620000000</v>
+        <v>0</v>
       </c>
       <c r="E10" s="12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13">
-        <v>240000000</v>
+        <v>0</v>
       </c>
       <c r="G10" s="12">
         <v>0</v>
@@ -4429,16 +4437,16 @@
         <v>0</v>
       </c>
       <c r="I10" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" s="13">
-        <v>110000000</v>
+        <v>0</v>
       </c>
       <c r="K10" s="12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13">
-        <v>130000000</v>
+        <v>0</v>
       </c>
       <c r="M10" s="12">
         <f>C10+E10+G10+I10+K10</f>
@@ -4479,10 +4487,10 @@
         <v>0</v>
       </c>
       <c r="K11" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L11" s="9">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="M11" s="8">
         <f>C11+E11+G11+I11+K11</f>
@@ -4651,7 +4659,7 @@
       <c r="I17" s="26"/>
       <c r="J17" s="26"/>
       <c r="K17" s="27">
-        <f>N12/N14</f>
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
       </c>
       <c r="L17" s="27"/>
     </row>
@@ -4672,7 +4680,7 @@
       <c r="I18" s="26"/>
       <c r="J18" s="26"/>
       <c r="K18" s="30">
-        <f>N13/N14</f>
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
       </c>
       <c r="L18" s="30"/>
     </row>
@@ -4733,6 +4741,640 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" s="3"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="8">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9">
+        <v>0</v>
+      </c>
+      <c r="K6" s="8">
+        <v>4</v>
+      </c>
+      <c r="L6" s="9">
+        <v>185000000</v>
+      </c>
+      <c r="M6" s="8">
+        <f>C6+E6+G6+I6+K6</f>
+      </c>
+      <c r="N6" s="9">
+        <f>D6+F6+H6+J6+L6</f>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>2</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="8">
+        <v>0</v>
+      </c>
+      <c r="D7" s="9">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9">
+        <v>0</v>
+      </c>
+      <c r="M7" s="8">
+        <f>C7+E7+G7+I7+K7</f>
+      </c>
+      <c r="N7" s="9">
+        <f>D7+F7+H7+J7+L7</f>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>3</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="8">
+        <v>0</v>
+      </c>
+      <c r="D8" s="9">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="9">
+        <v>0</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9">
+        <v>0</v>
+      </c>
+      <c r="K8" s="8">
+        <v>0</v>
+      </c>
+      <c r="L8" s="9">
+        <v>0</v>
+      </c>
+      <c r="M8" s="8">
+        <f>C8+E8+G8+I8+K8</f>
+      </c>
+      <c r="N8" s="9">
+        <f>D8+F8+H8+J8+L8</f>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>4</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="8">
+        <v>0</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0</v>
+      </c>
+      <c r="I9" s="8">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
+      <c r="K9" s="8">
+        <v>0</v>
+      </c>
+      <c r="L9" s="9">
+        <v>0</v>
+      </c>
+      <c r="M9" s="8">
+        <f>C9+E9+G9+I9+K9</f>
+      </c>
+      <c r="N9" s="9">
+        <f>D9+F9+H9+J9+L9</f>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="10">
+        <v>5</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="12">
+        <v>0</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+      <c r="E10" s="12">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0</v>
+      </c>
+      <c r="G10" s="12">
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
+        <v>0</v>
+      </c>
+      <c r="I10" s="12">
+        <v>0</v>
+      </c>
+      <c r="J10" s="13">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12">
+        <v>0</v>
+      </c>
+      <c r="L10" s="13">
+        <v>0</v>
+      </c>
+      <c r="M10" s="12">
+        <f>C10+E10+G10+I10+K10</f>
+      </c>
+      <c r="N10" s="13">
+        <f>D10+F10+H10+J10+L10</f>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>6</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="8">
+        <v>0</v>
+      </c>
+      <c r="D11" s="9">
+        <v>0</v>
+      </c>
+      <c r="E11" s="8">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9">
+        <v>0</v>
+      </c>
+      <c r="K11" s="8">
+        <v>0</v>
+      </c>
+      <c r="L11" s="9">
+        <v>0</v>
+      </c>
+      <c r="M11" s="8">
+        <f>C11+E11+G11+I11+K11</f>
+      </c>
+      <c r="N11" s="9">
+        <f>D11+F11+H11+J11+L11</f>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="14"/>
+      <c r="C12" s="15">
+        <f>C6+C7+C8+C9+C11</f>
+      </c>
+      <c r="D12" s="16">
+        <f>D6+D7+D8+D9+D11</f>
+      </c>
+      <c r="E12" s="15">
+        <f>E6+E7+E8+E9+E11</f>
+      </c>
+      <c r="F12" s="16">
+        <f>F6+F7+F8+F9+F11</f>
+      </c>
+      <c r="G12" s="15">
+        <f>G6+G7+G8+G9+G11</f>
+      </c>
+      <c r="H12" s="16">
+        <f>H6+H7+H8+H9+H11</f>
+      </c>
+      <c r="I12" s="15">
+        <f>I6+I7+I8+I9+I11</f>
+      </c>
+      <c r="J12" s="16">
+        <f>J6+J7+J8+J9+J11</f>
+      </c>
+      <c r="K12" s="15">
+        <f>K6+K7+K8+K9+K11</f>
+      </c>
+      <c r="L12" s="16">
+        <f>L6+L7+L8+L9+L11</f>
+      </c>
+      <c r="M12" s="15">
+        <f>M6+M7+M8+M9+M11</f>
+      </c>
+      <c r="N12" s="16">
+        <f>N6+N7+N8+N9+N11</f>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="18">
+        <f>C10</f>
+      </c>
+      <c r="D13" s="19">
+        <f>D10</f>
+      </c>
+      <c r="E13" s="18">
+        <f>E10</f>
+      </c>
+      <c r="F13" s="19">
+        <f>F10</f>
+      </c>
+      <c r="G13" s="18">
+        <f>G10</f>
+      </c>
+      <c r="H13" s="19">
+        <f>H10</f>
+      </c>
+      <c r="I13" s="18">
+        <f>I10</f>
+      </c>
+      <c r="J13" s="19">
+        <f>J10</f>
+      </c>
+      <c r="K13" s="18">
+        <f>K10</f>
+      </c>
+      <c r="L13" s="19">
+        <f>L10</f>
+      </c>
+      <c r="M13" s="18">
+        <f>M10</f>
+      </c>
+      <c r="N13" s="19">
+        <f>N10</f>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="21">
+        <f>C12+C13</f>
+      </c>
+      <c r="D14" s="22">
+        <f>D12+D13</f>
+      </c>
+      <c r="E14" s="21">
+        <f>E12+E13</f>
+      </c>
+      <c r="F14" s="22">
+        <f>F12+F13</f>
+      </c>
+      <c r="G14" s="21">
+        <f>G12+G13</f>
+      </c>
+      <c r="H14" s="22">
+        <f>H12+H13</f>
+      </c>
+      <c r="I14" s="21">
+        <f>I12+I13</f>
+      </c>
+      <c r="J14" s="22">
+        <f>J12+J13</f>
+      </c>
+      <c r="K14" s="21">
+        <f>K12+K13</f>
+      </c>
+      <c r="L14" s="22">
+        <f>L12+L13</f>
+      </c>
+      <c r="M14" s="21">
+        <f>M12+M13</f>
+      </c>
+      <c r="N14" s="22">
+        <f>N12+N13</f>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B16" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+    </row>
+    <row r="17" ht="24" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B17" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="25">
+        <f>N12</f>
+      </c>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="27">
+        <f>IF(N14&gt;0, N12/N14, 0)</f>
+      </c>
+      <c r="L17" s="27"/>
+    </row>
+    <row r="18" ht="24" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="29">
+        <f>N13</f>
+      </c>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="26" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" s="26"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="30">
+        <f>IF(N14&gt;0, N13/N14, 0)</f>
+      </c>
+      <c r="L18" s="30"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32">
+        <f>N14</f>
+      </c>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="I19" s="26"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="33">
+        <v>1</v>
+      </c>
+      <c r="L19" s="33"/>
+    </row>
+  </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="K19:L19"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -4744,7 +5386,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4752,100 +5394,100 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B3" s="34" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B5" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="36" t="s">
         <v>42</v>
-      </c>
-      <c r="C5" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="36" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" s="36" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D6" s="36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C7" s="36" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="35" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B9" s="36" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C9" s="36" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>